<commit_message>
feat: upgrade Excel dashboards with multi-tab structure, 12-week pilot tracking, v1 vs v2 matrix, and technical log dictionary
</commit_message>
<xml_diff>
--- a/v1/dashboard_hanh_dong_v1.xlsx
+++ b/v1/dashboard_hanh_dong_v1.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard_v1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard_v1_Activity" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nhan_Xet_Phan_Bien_Chieu" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,26 +30,50 @@
       <name val="Segoe UI"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="15"/>
+      <sz val="13"/>
     </font>
     <font>
       <name val="Segoe UI"/>
       <i val="1"/>
-      <color rgb="002C3E50"/>
-      <sz val="10"/>
+      <color rgb="00263238"/>
+      <sz val="9.5"/>
     </font>
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="10"/>
+      <sz val="9.5"/>
     </font>
     <font>
       <name val="Segoe UI"/>
-      <sz val="9.5"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <i val="1"/>
+      <color rgb="0037474F"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00263238"/>
+      <sz val="9"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -57,14 +82,38 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E78"/>
-        <bgColor rgb="001F4E78"/>
+        <fgColor rgb="00546E7A"/>
+        <bgColor rgb="00546E7A"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002F5597"/>
-        <bgColor rgb="002F5597"/>
+        <fgColor rgb="00ECEFF1"/>
+        <bgColor rgb="00ECEFF1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00455A64"/>
+        <bgColor rgb="00455A64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+        <bgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F7F9FB"/>
+        <bgColor rgb="00F7F9FB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0037474F"/>
+        <bgColor rgb="0037474F"/>
       </patternFill>
     </fill>
   </fills>
@@ -78,34 +127,58 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00BDC3C7"/>
+        <color rgb="00D0D7DE"/>
       </left>
       <right style="thin">
-        <color rgb="00BDC3C7"/>
+        <color rgb="00D0D7DE"/>
       </right>
       <top style="thin">
-        <color rgb="00BDC3C7"/>
+        <color rgb="00D0D7DE"/>
       </top>
       <bottom style="thin">
-        <color rgb="00BDC3C7"/>
+        <color rgb="00D0D7DE"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -476,38 +549,39 @@
   <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="25" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="35" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="36" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="35" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>DASHBOARD HÀNH ĐỘNG CHO ÁP DỤNG AI - BẢN V1 (TRƯỚC PHẢN BIỆN)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="22" customHeight="1">
+          <t>DASHBOARD HÀNH ĐỘNG CHO ÁP DỤNG AI (BẢN V1 - TRƯỚC PHẢN BIỆN CHÉO)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Case Study: Trợ lý AI tra cứu tài liệu &amp; chính sách nội bộ | Người dùng: Nhân viên Vận hành CSKH</t>
-        </is>
-      </c>
-    </row>
+          <t>Tình trạng: Bản sơ khởi ban đầu vướng bẫy 'Activity Metrics' (chỉ đếm lượt login, đếm câu hỏi, đo cảm tính)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Tầng đo lường / Loại chỉ số</t>
+          <t>Tầng đo lường (Dự kiến)</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Chỉ số cụ thể</t>
+          <t>Chỉ số ban đầu lựa chọn</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -522,21 +596,21 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Nguồn dữ liệu (Log/Hệ thống)</t>
+          <t>Nguồn dữ liệu</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Người phụ trách (Owner)</t>
+          <t>Người phụ trách</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Hành động khi chỉ số xấu</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="36" customHeight="1">
+          <t>Hành động dự kiến khi chỉ số xấu</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="38" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Tầng 1: Sử dụng (Activity)</t>
@@ -544,22 +618,22 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Số lượt đăng nhập vào hệ thống AI bot hàng tuần</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>45 lượt/tuần</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>&gt; 150 lượt/tuần</t>
+          <t>Số lượt đăng nhập vào hệ sinh thái AI bot hàng tuần</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>45 lượt / tuần</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>&gt; 150 lượt / tuần</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Log tài khoản SSO công ty</t>
+          <t>Log tài khoản SSO Google Workspace</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
@@ -569,48 +643,48 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>Gửi email nhắc nhở toàn công ty login</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="36" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
+          <t>Gửi email toàn công ty nhắc nhở mọi người đăng nhập dùng thử.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="38" customHeight="1">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>Tầng 1: Sử dụng (Activity)</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>Tổng số câu hỏi (prompt) gửi vào bot mỗi ngày</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>80 câu/ngày</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>&gt; 300 câu/ngày</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>Log chat server AI</t>
-        </is>
-      </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>80 câu / ngày</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>&gt; 300 câu / ngày</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>Log chat server AI nội bộ</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
         <is>
           <t>Nhóm dự án AI</t>
         </is>
       </c>
-      <c r="G6" s="4" t="inlineStr">
-        <is>
-          <t>Mở cuộc thi ai prompt nhiều nhất có thưởng</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="36" customHeight="1">
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>Tổ chức cuộc thi nhân viên nào prompt nhiều nhất trong tháng có thưởng voucher.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="38" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>Tầng 2: Hành vi</t>
@@ -621,19 +695,19 @@
           <t>Tỷ lệ nhân viên tham gia buổi đào tạo sử dụng bot</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>60%</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>100%</t>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>60% nhân viên</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>100% nhân viên</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Danh sách điểm danh HR</t>
+          <t>Danh sách điểm danh phòng HR</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
@@ -643,71 +717,71 @@
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>Tổ chức thêm lớp học bù bắt buộc</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="36" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>Tầng 3: Năng suất (Workflow)</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
+          <t>Tổ chức thêm 2 lớp học bù bắt buộc ngoài giờ cho các nhân viên vắng mặt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="38" customHeight="1">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Tầng 3: Năng suất (Tự khai)</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>Thời gian tiết kiệm ước tính theo người dùng tự khai</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>15 phút/ca</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>45 phút/ca</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>15 phút / ca</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>45 phút / ca</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
         <is>
           <t>Khảo sát Google Form cuối tháng</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="F8" s="6" t="inlineStr">
         <is>
           <t>Trưởng nhóm CSKH</t>
         </is>
       </c>
-      <c r="G8" s="4" t="inlineStr">
-        <is>
-          <t>Nhắc nhân viên trả lời khảo sát trung thực</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="36" customHeight="1">
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>Gửi tin nhắn Slack nhắc nhở nhân viên điền khảo sát nghiêm túc và trung thực.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="38" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Tầng 4: Chất lượng (Product)</t>
+          <t>Tầng 4: Chất lượng (Cảm tính)</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Độ chính xác câu trả lời theo đánh giá cảm tính</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>Chưa đo</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
+          <t>Mức độ hài lòng của nhân viên về câu trả lời của AI</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Chưa đo lường</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
         <is>
           <t>90% hài lòng</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Khảo sát 5 sao cuối câu trả lời</t>
+          <t>Khảo sát đánh giá 5 sao ở cuối mỗi câu trả lời bot</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
@@ -717,14 +791,163 @@
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>Xem xét lại prompt hệ thống</t>
+          <t>Họp với bên lập trình để xem lại cách viết prompt hệ thống.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>BIÊN BẢN GHI NHẬN PHẢN BIỆN CHÉO TẠI CHẶNG 3 (TỪ NHÓM 05)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>Các đóng góp xác đáng từ nhóm bạn giúp bản v1 lột xác thành bản v2 chuẩn quyết định</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4" ht="25" customHeight="1">
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>Trục đánh giá</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>Nhận xét của Nhóm 05 đối với bản v1</t>
+        </is>
+      </c>
+      <c r="C4" s="10" t="inlineStr">
+        <is>
+          <t>Khuyến nghị điều chỉnh</t>
+        </is>
+      </c>
+      <c r="D4" s="10" t="inlineStr">
+        <is>
+          <t>Kế hoạch khắc phục lên v2</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="45" customHeight="1">
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>1. Về chỉ số đo lường</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Bản v1 đang bị bẫy đếm số lượt login SSO và số câu prompt. Đây thuần túy là chỉ số hoạt động (Activity metric), không phản ánh việc nhân viên có làm nhanh hơn hay có giảm sai sót không.</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Loại bỏ login/prompt; thay bằng thời gian xử lý ca đo từ log Jira và tỷ lệ trả lời có trích dẫn nguồn kiểm chứng được.</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Đã nâng cấp thành M03_CYCLE_TIME và M04_CITE_ACC trong bản v2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="45" customHeight="1">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>2. Về tính xác thực dữ liệu</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>Thời gian tiết kiệm lấy từ Google Form tự khai là không đáng tin cậy vì nhân viên có xu hướng khai khống hoặc khai đại.</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>Bắt buộc lấy timestamp trực tiếp từ hệ thống quản lý tác vụ (Ticket resolution time).</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>Đã tích hợp API log của Jira Service Management vào từ điển dữ liệu Tab 4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="45" customHeight="1">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>3. Về giải pháp đào tạo</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Cột hành động khi chỉ số xấu chỉ đề xuất 'mở thêm lớp học bù' là quá thô sơ. Vấn đề nằm ở việc nhân viên sợ AI trả lời sai dẫn đến đền tiền.</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Cần xây dựng cơ chế kiểm soát chất lượng (Trust Architecture) và chính sách miễn trừ trách nhiệm theo Mollick.</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Đã thiết lập quy trình TO-BE có trích nguồn + nút báo lỗi + bảo vệ nhân viên tại Memo và Dashboard v2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="45" customHeight="1">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>4. Về phân công Owner</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>Người phụ trách ghi chung chung là 'IT Admin' hoặc 'Nhóm AI' là chưa đúng với bản chất quy trình nghiệp vụ.</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>Mỗi chỉ số phải có Chủ quy trình nghiệp vụ (Process Owner) hoặc Quản lý ca đứng tên chịu trách nhiệm.</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>Đã phân công đích danh: Chủ quy trình CSKH, Trưởng phòng CSKH, QA Lead, COO.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>